<commit_message>
docs: upload records of 2 interviews #23
</commit_message>
<xml_diff>
--- a/docs/surveys/answer_form.xlsx
+++ b/docs/surveys/answer_form.xlsx
@@ -1,33 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10907"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b8827725017ffd42/Documents/GitHub/software-AI66B-G2-B4-small-shop/docs/surveys/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{396089A5-FCDF-4E80-9446-46B54DFD2512}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DFD9DB7-1166-9841-BD1E-0ED7AF9FB2A1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet3 (2)" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet3 (3)" sheetId="5" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="19">
   <si>
     <t>Interviewee info</t>
   </si>
@@ -63,6 +76,27 @@
   </si>
   <si>
     <t>Further discussions</t>
+  </si>
+  <si>
+    <t>Mỹ đoan</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Cáchao thao tác ỏtreen app</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chia mục riêng, tạo sẵn size, đươgf đá, note </t>
+  </si>
+  <si>
+    <t>Doanh thu</t>
+  </si>
+  <si>
+    <t>Xem theo ngày, ipos chia m</t>
+  </si>
+  <si>
+    <t>Chia ca</t>
   </si>
 </sst>
 </file>
@@ -73,7 +107,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -81,14 +115,14 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -142,7 +176,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -155,10 +189,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -425,20 +455,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="33.5546875" style="2" customWidth="1"/>
-    <col min="3" max="5" width="8.88671875" style="2"/>
-    <col min="6" max="6" width="35.77734375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="35.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="26.33203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="2"/>
-    <col min="10" max="10" width="18.21875" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="17.40625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.58984375" style="2" customWidth="1"/>
+    <col min="3" max="5" width="8.82421875" style="2"/>
+    <col min="6" max="6" width="35.796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="35.671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="26.35546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="8.82421875" style="2"/>
+    <col min="10" max="10" width="18.265625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.82421875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -446,11 +476,13 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
+      <c r="B3" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
@@ -464,37 +496,49 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="3"/>
       <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="3"/>
       <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
@@ -504,7 +548,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
@@ -514,85 +558,85 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
     </row>
-    <row r="18" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
-    <row r="19" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -606,20 +650,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A217A6C-524B-4203-A4A6-6CA5EAD09804}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="33.5546875" style="2" customWidth="1"/>
-    <col min="3" max="5" width="8.88671875" style="2"/>
-    <col min="6" max="6" width="35.77734375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="35.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="26.33203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="2"/>
-    <col min="10" max="10" width="18.21875" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="17.40625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.58984375" style="2" customWidth="1"/>
+    <col min="3" max="5" width="8.82421875" style="2"/>
+    <col min="6" max="6" width="35.796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="35.671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="26.35546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="8.82421875" style="2"/>
+    <col min="10" max="10" width="18.265625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.82421875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -627,7 +671,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -645,7 +689,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -655,7 +699,7 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
@@ -665,7 +709,7 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
@@ -675,7 +719,7 @@
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
@@ -685,7 +729,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
@@ -695,85 +739,85 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
     </row>
-    <row r="18" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
-    <row r="19" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -785,22 +829,22 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BE72C04-0EC7-4EF0-9167-5142F00B9805}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D1157F1-6914-0848-A430-FCE90E931F4E}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="33.5546875" style="2" customWidth="1"/>
-    <col min="3" max="5" width="8.88671875" style="2"/>
-    <col min="6" max="6" width="35.77734375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="35.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="26.33203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="2"/>
-    <col min="10" max="10" width="18.21875" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="17.40625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.58984375" style="2" customWidth="1"/>
+    <col min="3" max="5" width="8.82421875" style="2"/>
+    <col min="6" max="6" width="35.796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="35.671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="26.35546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="8.82421875" style="2"/>
+    <col min="10" max="10" width="18.265625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.82421875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -808,7 +852,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -826,7 +870,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -836,7 +880,7 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
@@ -846,7 +890,7 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
@@ -856,7 +900,7 @@
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
@@ -866,7 +910,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
@@ -876,85 +920,85 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
     </row>
-    <row r="18" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
-    <row r="19" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:8" x14ac:dyDescent="0.15">
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -963,4 +1007,366 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1755AC25-5271-AE45-8EB1-D72D4D78ABA5}">
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="17.40625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.58984375" style="2" customWidth="1"/>
+    <col min="3" max="5" width="8.82421875" style="2"/>
+    <col min="6" max="6" width="35.796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="35.671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="26.35546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="8.82421875" style="2"/>
+    <col min="10" max="10" width="18.265625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.82421875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="E3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BE72C04-0EC7-4EF0-9167-5142F00B9805}">
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="17.40625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.58984375" style="2" customWidth="1"/>
+    <col min="3" max="5" width="8.82421875" style="2"/>
+    <col min="6" max="6" width="35.796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="35.671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="26.35546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="8.82421875" style="2"/>
+    <col min="10" max="10" width="18.265625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.82421875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="E3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: transcript 3rd interview #24
Refs #24
</commit_message>
<xml_diff>
--- a/docs/surveys/answer_form.xlsx
+++ b/docs/surveys/answer_form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b8827725017ffd42/Documents/GitHub/software-AI66B-G2-B4-small-shop/docs/surveys/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="209" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB3B8852-106D-4BFC-9EFF-B5DB5AE34BCE}"/>
+  <xr:revisionPtr revIDLastSave="273" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AB493CF-EBBE-4F03-A61C-67833543C1C8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="124">
   <si>
     <t>Interviewee info</t>
   </si>
@@ -46,9 +46,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Birth year</t>
-  </si>
-  <si>
     <t>Shop name</t>
   </si>
   <si>
@@ -317,13 +314,109 @@
   </si>
   <si>
     <t>a growing family-business banh trang brand has opened a few branches around Hanoi. They have a lot of customer, yet just 2 owners and 3 other employees working in the shop the entire day. They sell both take away, dine-in and digital apps (grab, shopee,...). their demand in managing is not too high or complicated. keeping both physical notebooks and an selling app to track the income (revenue)</t>
+  </si>
+  <si>
+    <t>Linh</t>
+  </si>
+  <si>
+    <t>Employee - Cashier</t>
+  </si>
+  <si>
+    <t>Ớt Chuông Mart</t>
+  </si>
+  <si>
+    <t>235 Đội Cấn</t>
+  </si>
+  <si>
+    <t>processed food (frozen, canned, packaged,... Litterally the things you can find in a supermart)</t>
+  </si>
+  <si>
+    <t>take away</t>
+  </si>
+  <si>
+    <t>a retain chain consists of small supermarkets around Hanoi, managed by a team of small yet professional company. They sell mostly processed food, frozen food, snacks,… and some other home appliances. Their products are special because they can barely be seen in mainstream retailers. the managing process requires professional, sequential tasks, reports.</t>
+  </si>
+  <si>
+    <t>When you open a shift and start taking orders on the store app, what is your exact workflow?</t>
+  </si>
+  <si>
+    <t>You mentioned searching for customer profiles by phone number. How does that customer tracking feature work on your app?</t>
+  </si>
+  <si>
+    <t>Can you see or edit customer details beyond just adding points, or check overall customer analytics?</t>
+  </si>
+  <si>
+    <t>If a customer changes their phone number or wants to fix their name, I can't update it on my end. I have to write it down on a sticky note for the store manager to fix later.</t>
+  </si>
+  <si>
+    <t>Does the app allow you to see or manage store inventory or revenues?</t>
+  </si>
+  <si>
+    <t>Since the app doesn't show revenue or inventory to cashiers, how do you handle shift handovers and reporting at the end of the day?</t>
+  </si>
+  <si>
+    <t>How are staff attendance, shift scheduling, and individual employee performance tracked in your shop?</t>
+  </si>
+  <si>
+    <t>What do you think are the biggest advantages of using this managing app in your daily routine?</t>
+  </si>
+  <si>
+    <t>If the app added an AI feature to recommend up-sell items to customers at checkout based on their profile (e.g., suggesting a complementary sauce for frozen food), would you use it?</t>
+  </si>
+  <si>
+    <t>First I log into my assigned cashier account—we have individual log-ins here. When a customer brings items to the counter, I scan the barcodes using the attached scanner or search by item name or category code. After scanning, I ask for their phone number to log their loyalty account, pick the payment method, cash out, and print the receipt.</t>
+  </si>
+  <si>
+    <t>We just type in their phone number. If they are already in the system, it pulls up their name, current reward points, and purchase history. If they’re new, I would ask for their names and add into the system. Every order automatically adds points to their profile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">but if there's a long queue, asking every single customer for their phone number would take lots of time and the waiting customer would be mad and make complaints. </t>
+  </si>
+  <si>
+    <t>No, i can only see profiles. The points are added automatically during checkout and base on orders. We can't edit personal details.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. but We can see stock counts. </t>
+  </si>
+  <si>
+    <t>but in the end of the day, I some times have to assist the manager in checking the stocks. She will write down the stocks in a paper form.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At the end of my shift, i just put my finger in the checking attendance machine, log out of the app. I don’t have to do reports. The manager can check my KPI at the end of the day. </t>
+  </si>
+  <si>
+    <t>They are very strict here. If the physical cash drawer is even 10,000 VND short compared to the app report, we will be asked and required to explain right away. Mostly directly or through a group chat on Zalo.</t>
+  </si>
+  <si>
+    <t>Attendance is done via fingerprint scanner at the entrance, not through this sales app. But the app tracks sales per cashier account.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It’s very structured and hard to make mistakes with pricing or product names. The names here are weird, but we can search quickly. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">but it required tranning. I still feel struggled some times. </t>
+  </si>
+  <si>
+    <t>what are the main drawbacks or frustrations you experience while using the app?</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> there are minor lags.</t>
+  </si>
+  <si>
+    <t>can you suggest improvements for the app to make your job easier?</t>
+  </si>
+  <si>
+    <t>small cashier dashboard showing our own daily stats,  for personal tracking.</t>
+  </si>
+  <si>
+    <t>maybe like 60-70%. It could be helpful for new staff. But most customers come in with a very specific shopping list and just want to pay and leave quickly. If I push extra recommendations, it might slow down the line and annoy them.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -346,6 +439,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -361,7 +469,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -384,11 +492,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -404,6 +551,27 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -689,7 +857,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.88671875" style="2" customWidth="1"/>
@@ -708,7 +876,7 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -716,133 +884,133 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" s="4">
         <v>1</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" s="4">
         <v>2</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E6" s="4">
         <v>3</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" s="4">
         <v>4</v>
       </c>
       <c r="F7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>18</v>
       </c>
       <c r="E8" s="4">
         <v>5</v>
       </c>
       <c r="F8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>60</v>
       </c>
       <c r="E9" s="4">
         <v>6</v>
       </c>
       <c r="F9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G9" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="H9" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
@@ -850,10 +1018,10 @@
         <v>7</v>
       </c>
       <c r="F10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="H10" s="4"/>
     </row>
@@ -862,13 +1030,13 @@
         <v>8</v>
       </c>
       <c r="F11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
@@ -876,13 +1044,13 @@
         <v>9</v>
       </c>
       <c r="F12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="H12" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
@@ -890,13 +1058,13 @@
         <v>10</v>
       </c>
       <c r="F13" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="H13" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="124.8" x14ac:dyDescent="0.3">
@@ -904,10 +1072,10 @@
         <v>11</v>
       </c>
       <c r="F14" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>46</v>
       </c>
       <c r="H14" s="4"/>
     </row>
@@ -916,10 +1084,10 @@
         <v>12</v>
       </c>
       <c r="F15" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="H15" s="4"/>
     </row>
@@ -928,10 +1096,10 @@
         <v>13</v>
       </c>
       <c r="F16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="H16" s="4"/>
     </row>
@@ -940,13 +1108,13 @@
         <v>14</v>
       </c>
       <c r="F17" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="H17" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="18" spans="5:8" ht="46.8" x14ac:dyDescent="0.3">
@@ -954,13 +1122,13 @@
         <v>15</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G18" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H18" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="19" spans="5:8" ht="31.2" x14ac:dyDescent="0.3">
@@ -968,24 +1136,12 @@
         <v>16</v>
       </c>
       <c r="F19" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G19" s="4" t="s">
-        <v>56</v>
-      </c>
       <c r="H19" s="4"/>
-    </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -995,7 +1151,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A217A6C-524B-4203-A4A6-6CA5EAD09804}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.77734375" style="2" customWidth="1"/>
@@ -1014,7 +1170,7 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1022,129 +1178,129 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E4" s="4">
         <v>1</v>
       </c>
       <c r="F4" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E5" s="4">
         <v>2</v>
       </c>
       <c r="F5" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>70</v>
       </c>
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E6" s="4">
         <v>3</v>
       </c>
       <c r="F6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E7" s="4">
         <v>4</v>
       </c>
       <c r="F7" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>74</v>
       </c>
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E8" s="4">
         <v>5</v>
       </c>
       <c r="F8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="202.8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E9" s="4">
         <v>6</v>
       </c>
       <c r="F9" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
@@ -1152,10 +1308,10 @@
         <v>7</v>
       </c>
       <c r="F10" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>81</v>
       </c>
       <c r="H10" s="4"/>
     </row>
@@ -1164,10 +1320,10 @@
         <v>8</v>
       </c>
       <c r="F11" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="H11" s="4"/>
     </row>
@@ -1176,10 +1332,10 @@
         <v>9</v>
       </c>
       <c r="F12" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="H12" s="4"/>
     </row>
@@ -1188,10 +1344,10 @@
         <v>10</v>
       </c>
       <c r="F13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>87</v>
       </c>
       <c r="H13" s="4"/>
     </row>
@@ -1200,10 +1356,10 @@
         <v>11</v>
       </c>
       <c r="F14" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="H14" s="4"/>
     </row>
@@ -1212,54 +1368,12 @@
         <v>12</v>
       </c>
       <c r="F15" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="G15" s="4" t="s">
-        <v>91</v>
-      </c>
       <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-    </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-    </row>
-    <row r="18" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-    </row>
-    <row r="19" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-    </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-    </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1268,187 +1382,298 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D1157F1-6914-0848-A430-FCE90E931F4E}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.77734375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="33.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="42.33203125" style="2" customWidth="1"/>
     <col min="3" max="5" width="8.77734375" style="2"/>
     <col min="6" max="6" width="35.77734375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="35.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="26.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="50.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="50.109375" style="2" customWidth="1"/>
     <col min="9" max="9" width="8.77734375" style="2"/>
     <col min="10" max="10" width="18.21875" style="2" customWidth="1"/>
     <col min="11" max="16384" width="8.77734375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="E3" s="3" t="s">
+      <c r="B3" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="7">
+        <v>1</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="H4" s="8"/>
+    </row>
+    <row r="5" spans="1:9" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" s="7">
+        <v>2</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="7">
         <v>3</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-    </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F6" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="7">
+        <v>4</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="78" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" s="7">
+        <v>5</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="156" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="7">
         <v>6</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-    </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
+      <c r="F9" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>116</v>
+      </c>
       <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" s="2" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-    </row>
-    <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="17" spans="5:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="5:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-    </row>
-    <row r="19" spans="5:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" spans="5:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-    </row>
-    <row r="21" spans="5:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-    </row>
-    <row r="22" spans="5:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:9" ht="85.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E10" s="7">
+        <v>7</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="E11" s="7">
+        <v>8</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="H11" s="8"/>
+    </row>
+    <row r="12" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="E12" s="7">
+        <v>9</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="H12" s="8"/>
+    </row>
+    <row r="13" spans="1:9" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="E13" s="7">
+        <v>10</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H13" s="8"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+    </row>
+    <row r="17" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+    </row>
+    <row r="18" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+    </row>
+    <row r="19" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+    </row>
+    <row r="20" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+    </row>
+    <row r="21" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+    </row>
+    <row r="22" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+    </row>
+    <row r="23" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+    </row>
+    <row r="24" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+    </row>
+    <row r="25" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: wrote product visions and personas
Refs #36 #37
</commit_message>
<xml_diff>
--- a/docs/surveys/answer_form.xlsx
+++ b/docs/surveys/answer_form.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b8827725017ffd42/Documents/GitHub/software-AI66B-G2-B4-small-shop/docs/surveys/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="273" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AB493CF-EBBE-4F03-A61C-67833543C1C8}"/>
+  <xr:revisionPtr revIDLastSave="274" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC1AE83F-28DE-4733-B478-C0890C04BF89}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="My Doan (RR)" sheetId="1" r:id="rId1"/>
     <sheet name="Viet (BTBM)" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3 (2)" sheetId="4" r:id="rId3"/>
+    <sheet name="Linh (OTM)" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -535,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -547,9 +547,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -567,7 +564,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1382,7 +1379,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D1157F1-6914-0848-A430-FCE90E931F4E}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.77734375" style="2" customWidth="1"/>
@@ -1411,36 +1408,36 @@
       <c r="B3" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="6">
         <v>1</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="8"/>
+      <c r="H4" s="7"/>
     </row>
     <row r="5" spans="1:9" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -1449,16 +1446,16 @@
       <c r="B5" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <v>2</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="7" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1469,16 +1466,16 @@
       <c r="B6" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="6">
         <v>3</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="7" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1489,16 +1486,16 @@
       <c r="B7" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <v>4</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="7" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1509,16 +1506,16 @@
       <c r="B8" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <v>5</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="8" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1529,151 +1526,67 @@
       <c r="B9" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="6">
         <v>6</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="9" t="s">
         <v>116</v>
       </c>
       <c r="H9" s="4"/>
-      <c r="I9" s="11"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:9" ht="85.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E10" s="7">
+      <c r="E10" s="6">
         <v>7</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="11" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="E11" s="7">
+      <c r="E11" s="6">
         <v>8</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="H11" s="8"/>
+      <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="E12" s="7">
+      <c r="E12" s="6">
         <v>9</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="H12" s="8"/>
+      <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:9" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="E13" s="7">
+      <c r="E13" s="6">
         <v>10</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="H13" s="8"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-    </row>
-    <row r="17" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-    </row>
-    <row r="18" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-    </row>
-    <row r="19" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-    </row>
-    <row r="20" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-    </row>
-    <row r="21" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-    </row>
-    <row r="22" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-    </row>
-    <row r="23" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-    </row>
-    <row r="24" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-    </row>
-    <row r="25" spans="5:9" x14ac:dyDescent="0.3">
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
+      <c r="H13" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>